<commit_message>
feat(proposals): institution directory search, batch co-investigator invites, budget preview
</commit_message>
<xml_diff>
--- a/Claude outputs/sample-project-joy-owango/TRIAGE-KE_Budget.xlsx
+++ b/Claude outputs/sample-project-joy-owango/TRIAGE-KE_Budget.xlsx
@@ -127,7 +127,7 @@
     <t xml:space="preserve">Project duration (months)</t>
   </si>
   <si>
-    <t xml:space="preserve">Proposal: 1 Oct 2025 – 31 Mar 2027</t>
+    <t xml:space="preserve">Proposal: 25 Oct 2026 – 24 Apr 2028</t>
   </si>
   <si>
     <t xml:space="preserve">Indirect cost rate (on direct costs)</t>
@@ -163,7 +163,7 @@
     <t xml:space="preserve">TRIAGE-KE — Detailed Budget (KES)</t>
   </si>
   <si>
-    <t xml:space="preserve">PI: Joy Owango · Grant HDHIF/2025/017 · Funder: Hospitium Digital Health Innovation Fund (Demo) · SAMPLE DATA</t>
+    <t xml:space="preserve">PI: Joy Owango · Grant HDHIF/2026/017 · Funder: Hospitium Digital Health Innovation Fund (Demo) · SAMPLE DATA</t>
   </si>
   <si>
     <t xml:space="preserve">Code</t>
@@ -256,7 +256,7 @@
     <t xml:space="preserve">Research Assistants (2 per site)</t>
   </si>
   <si>
-    <t xml:space="preserve">Data abstraction &amp; observation, Nov 2025 – Jul 2026</t>
+    <t xml:space="preserve">Data abstraction &amp; observation, Dec 2026 – Aug 2027</t>
   </si>
   <si>
     <t xml:space="preserve">A8</t>
@@ -502,7 +502,7 @@
     <t xml:space="preserve">Conference attendance (regional)</t>
   </si>
   <si>
-    <t xml:space="preserve">Abstract presentation, 2027</t>
+    <t xml:space="preserve">Abstract presentation, 2028</t>
   </si>
   <si>
     <t xml:space="preserve">G3</t>
@@ -556,7 +556,7 @@
     <t xml:space="preserve">TOTAL DIRECT COSTS</t>
   </si>
   <si>
-    <t xml:space="preserve">Note: Year 1 = Oct 2025 – Sep 2026; Year 2 = Oct 2026 – Mar 2027. Year-1 share is an input per line.</t>
+    <t xml:space="preserve">Note: Year 1 = 25 Oct 2026 – 24 Oct 2027; Year 2 = 25 Oct 2027 – 24 Apr 2028. Year-1 share is an input per line.</t>
   </si>
 </sst>
 </file>

</xml_diff>